<commit_message>
Pushing some CAD updates and assets
</commit_message>
<xml_diff>
--- a/Projektmanagement_Gantt-Diagramm.xlsx
+++ b/Projektmanagement_Gantt-Diagramm.xlsx
@@ -1286,9 +1286,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1904040</xdr:colOff>
+      <xdr:colOff>1903680</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>523080</xdr:rowOff>
+      <xdr:rowOff>522720</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1304,7 +1304,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="95400"/>
-          <a:ext cx="1904040" cy="427680"/>
+          <a:ext cx="1903680" cy="427320"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1570,11 +1570,11 @@
       </c>
       <c r="D5" s="17"/>
       <c r="E5" s="19" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="I5" s="20" t="n">
         <f aca="false">I6</f>
-        <v>46020</v>
+        <v>46055</v>
       </c>
       <c r="J5" s="20"/>
       <c r="K5" s="20"/>
@@ -1584,7 +1584,7 @@
       <c r="O5" s="20"/>
       <c r="P5" s="20" t="n">
         <f aca="false">P6</f>
-        <v>46027</v>
+        <v>46062</v>
       </c>
       <c r="Q5" s="20"/>
       <c r="R5" s="20"/>
@@ -1594,7 +1594,7 @@
       <c r="V5" s="20"/>
       <c r="W5" s="20" t="n">
         <f aca="false">W6</f>
-        <v>46034</v>
+        <v>46069</v>
       </c>
       <c r="X5" s="20"/>
       <c r="Y5" s="20"/>
@@ -1604,7 +1604,7 @@
       <c r="AC5" s="20"/>
       <c r="AD5" s="20" t="n">
         <f aca="false">AD6</f>
-        <v>46041</v>
+        <v>46076</v>
       </c>
       <c r="AE5" s="20"/>
       <c r="AF5" s="20"/>
@@ -1614,7 +1614,7 @@
       <c r="AJ5" s="20"/>
       <c r="AK5" s="20" t="n">
         <f aca="false">AK6</f>
-        <v>46048</v>
+        <v>46083</v>
       </c>
       <c r="AL5" s="20"/>
       <c r="AM5" s="20"/>
@@ -1624,7 +1624,7 @@
       <c r="AQ5" s="20"/>
       <c r="AR5" s="20" t="n">
         <f aca="false">AR6</f>
-        <v>46055</v>
+        <v>46090</v>
       </c>
       <c r="AS5" s="20"/>
       <c r="AT5" s="20"/>
@@ -1634,7 +1634,7 @@
       <c r="AX5" s="20"/>
       <c r="AY5" s="20" t="n">
         <f aca="false">AY6</f>
-        <v>46062</v>
+        <v>46097</v>
       </c>
       <c r="AZ5" s="20"/>
       <c r="BA5" s="20"/>
@@ -1644,7 +1644,7 @@
       <c r="BE5" s="20"/>
       <c r="BF5" s="20" t="n">
         <f aca="false">BF6</f>
-        <v>46069</v>
+        <v>46104</v>
       </c>
       <c r="BG5" s="20"/>
       <c r="BH5" s="20"/>
@@ -1665,227 +1665,227 @@
       <c r="G6" s="21"/>
       <c r="I6" s="22" t="n">
         <f aca="false">Projektanfang-WEEKDAY(Projektanfang,1)+2+7*(Anzeigewoche-1)</f>
-        <v>46020</v>
+        <v>46055</v>
       </c>
       <c r="J6" s="23" t="n">
         <f aca="false">I6+1</f>
-        <v>46021</v>
+        <v>46056</v>
       </c>
       <c r="K6" s="23" t="n">
         <f aca="false">J6+1</f>
-        <v>46022</v>
+        <v>46057</v>
       </c>
       <c r="L6" s="23" t="n">
         <f aca="false">K6+1</f>
-        <v>46023</v>
+        <v>46058</v>
       </c>
       <c r="M6" s="23" t="n">
         <f aca="false">L6+1</f>
-        <v>46024</v>
+        <v>46059</v>
       </c>
       <c r="N6" s="23" t="n">
         <f aca="false">M6+1</f>
-        <v>46025</v>
+        <v>46060</v>
       </c>
       <c r="O6" s="24" t="n">
         <f aca="false">N6+1</f>
-        <v>46026</v>
+        <v>46061</v>
       </c>
       <c r="P6" s="22" t="n">
         <f aca="false">O6+1</f>
-        <v>46027</v>
+        <v>46062</v>
       </c>
       <c r="Q6" s="23" t="n">
         <f aca="false">P6+1</f>
-        <v>46028</v>
+        <v>46063</v>
       </c>
       <c r="R6" s="23" t="n">
         <f aca="false">Q6+1</f>
-        <v>46029</v>
+        <v>46064</v>
       </c>
       <c r="S6" s="23" t="n">
         <f aca="false">R6+1</f>
-        <v>46030</v>
+        <v>46065</v>
       </c>
       <c r="T6" s="23" t="n">
         <f aca="false">S6+1</f>
-        <v>46031</v>
+        <v>46066</v>
       </c>
       <c r="U6" s="23" t="n">
         <f aca="false">T6+1</f>
-        <v>46032</v>
+        <v>46067</v>
       </c>
       <c r="V6" s="24" t="n">
         <f aca="false">U6+1</f>
-        <v>46033</v>
+        <v>46068</v>
       </c>
       <c r="W6" s="22" t="n">
         <f aca="false">V6+1</f>
-        <v>46034</v>
+        <v>46069</v>
       </c>
       <c r="X6" s="23" t="n">
         <f aca="false">W6+1</f>
-        <v>46035</v>
+        <v>46070</v>
       </c>
       <c r="Y6" s="23" t="n">
         <f aca="false">X6+1</f>
-        <v>46036</v>
+        <v>46071</v>
       </c>
       <c r="Z6" s="23" t="n">
         <f aca="false">Y6+1</f>
-        <v>46037</v>
+        <v>46072</v>
       </c>
       <c r="AA6" s="23" t="n">
         <f aca="false">Z6+1</f>
-        <v>46038</v>
+        <v>46073</v>
       </c>
       <c r="AB6" s="23" t="n">
         <f aca="false">AA6+1</f>
-        <v>46039</v>
+        <v>46074</v>
       </c>
       <c r="AC6" s="24" t="n">
         <f aca="false">AB6+1</f>
-        <v>46040</v>
+        <v>46075</v>
       </c>
       <c r="AD6" s="22" t="n">
         <f aca="false">AC6+1</f>
-        <v>46041</v>
+        <v>46076</v>
       </c>
       <c r="AE6" s="23" t="n">
         <f aca="false">AD6+1</f>
-        <v>46042</v>
+        <v>46077</v>
       </c>
       <c r="AF6" s="23" t="n">
         <f aca="false">AE6+1</f>
-        <v>46043</v>
+        <v>46078</v>
       </c>
       <c r="AG6" s="23" t="n">
         <f aca="false">AF6+1</f>
-        <v>46044</v>
+        <v>46079</v>
       </c>
       <c r="AH6" s="23" t="n">
         <f aca="false">AG6+1</f>
-        <v>46045</v>
+        <v>46080</v>
       </c>
       <c r="AI6" s="23" t="n">
         <f aca="false">AH6+1</f>
-        <v>46046</v>
+        <v>46081</v>
       </c>
       <c r="AJ6" s="24" t="n">
         <f aca="false">AI6+1</f>
-        <v>46047</v>
+        <v>46082</v>
       </c>
       <c r="AK6" s="22" t="n">
         <f aca="false">AJ6+1</f>
-        <v>46048</v>
+        <v>46083</v>
       </c>
       <c r="AL6" s="23" t="n">
         <f aca="false">AK6+1</f>
-        <v>46049</v>
+        <v>46084</v>
       </c>
       <c r="AM6" s="23" t="n">
         <f aca="false">AL6+1</f>
-        <v>46050</v>
+        <v>46085</v>
       </c>
       <c r="AN6" s="23" t="n">
         <f aca="false">AM6+1</f>
-        <v>46051</v>
+        <v>46086</v>
       </c>
       <c r="AO6" s="23" t="n">
         <f aca="false">AN6+1</f>
-        <v>46052</v>
+        <v>46087</v>
       </c>
       <c r="AP6" s="23" t="n">
         <f aca="false">AO6+1</f>
-        <v>46053</v>
+        <v>46088</v>
       </c>
       <c r="AQ6" s="24" t="n">
         <f aca="false">AP6+1</f>
-        <v>46054</v>
+        <v>46089</v>
       </c>
       <c r="AR6" s="22" t="n">
         <f aca="false">AQ6+1</f>
-        <v>46055</v>
+        <v>46090</v>
       </c>
       <c r="AS6" s="23" t="n">
         <f aca="false">AR6+1</f>
-        <v>46056</v>
+        <v>46091</v>
       </c>
       <c r="AT6" s="23" t="n">
         <f aca="false">AS6+1</f>
-        <v>46057</v>
+        <v>46092</v>
       </c>
       <c r="AU6" s="23" t="n">
         <f aca="false">AT6+1</f>
-        <v>46058</v>
+        <v>46093</v>
       </c>
       <c r="AV6" s="23" t="n">
         <f aca="false">AU6+1</f>
-        <v>46059</v>
+        <v>46094</v>
       </c>
       <c r="AW6" s="23" t="n">
         <f aca="false">AV6+1</f>
-        <v>46060</v>
+        <v>46095</v>
       </c>
       <c r="AX6" s="24" t="n">
         <f aca="false">AW6+1</f>
-        <v>46061</v>
+        <v>46096</v>
       </c>
       <c r="AY6" s="22" t="n">
         <f aca="false">AX6+1</f>
-        <v>46062</v>
+        <v>46097</v>
       </c>
       <c r="AZ6" s="23" t="n">
         <f aca="false">AY6+1</f>
-        <v>46063</v>
+        <v>46098</v>
       </c>
       <c r="BA6" s="23" t="n">
         <f aca="false">AZ6+1</f>
-        <v>46064</v>
+        <v>46099</v>
       </c>
       <c r="BB6" s="23" t="n">
         <f aca="false">BA6+1</f>
-        <v>46065</v>
+        <v>46100</v>
       </c>
       <c r="BC6" s="23" t="n">
         <f aca="false">BB6+1</f>
-        <v>46066</v>
+        <v>46101</v>
       </c>
       <c r="BD6" s="23" t="n">
         <f aca="false">BC6+1</f>
-        <v>46067</v>
+        <v>46102</v>
       </c>
       <c r="BE6" s="24" t="n">
         <f aca="false">BD6+1</f>
-        <v>46068</v>
+        <v>46103</v>
       </c>
       <c r="BF6" s="22" t="n">
         <f aca="false">BE6+1</f>
-        <v>46069</v>
+        <v>46104</v>
       </c>
       <c r="BG6" s="23" t="n">
         <f aca="false">BF6+1</f>
-        <v>46070</v>
+        <v>46105</v>
       </c>
       <c r="BH6" s="23" t="n">
         <f aca="false">BG6+1</f>
-        <v>46071</v>
+        <v>46106</v>
       </c>
       <c r="BI6" s="23" t="n">
         <f aca="false">BH6+1</f>
-        <v>46072</v>
+        <v>46107</v>
       </c>
       <c r="BJ6" s="23" t="n">
         <f aca="false">BI6+1</f>
-        <v>46073</v>
+        <v>46108</v>
       </c>
       <c r="BK6" s="23" t="n">
         <f aca="false">BJ6+1</f>
-        <v>46074</v>
+        <v>46109</v>
       </c>
       <c r="BL6" s="24" t="n">
         <f aca="false">BK6+1</f>
-        <v>46075</v>
+        <v>46110</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2288,7 +2288,7 @@
         <v>5</v>
       </c>
       <c r="D10" s="39" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="E10" s="40" t="n">
         <v>46106</v>
@@ -2439,7 +2439,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="39" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="E12" s="40" t="n">
         <v>46106</v>
@@ -2513,7 +2513,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="39" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E13" s="40" t="n">
         <v>46106</v>
@@ -4921,7 +4921,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D44F12C0-524D-4E10-AB61-98EB6665C14B}</x14:id>
+          <x14:id>{DA70804D-8188-4E2D-B444-C34A4E7E1947}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4962,7 +4962,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D44F12C0-524D-4E10-AB61-98EB6665C14B}">
+          <x14:cfRule type="dataBar" id="{DA70804D-8188-4E2D-B444-C34A4E7E1947}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="automatic" gradient="false">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5032,7 +5032,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="74.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="92" t="s">
         <v>58</v>
       </c>
@@ -5067,7 +5067,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="74.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="92" t="s">
         <v>65</v>
       </c>

</xml_diff>

<commit_message>
Remove old CAD Files not needed anymore
</commit_message>
<xml_diff>
--- a/Projektmanagement_Gantt-Diagramm.xlsx
+++ b/Projektmanagement_Gantt-Diagramm.xlsx
@@ -1,38 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_58D18C6C6B7024444B3B59DB4C5A0E8A8BD3A42C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="7"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Projektplan" sheetId="1" r:id="rId1"/>
-    <sheet name="Info" sheetId="2" r:id="rId2"/>
+    <sheet name="Projektplan" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Info" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="Anzeigewoche">Projektplan!$E$5</definedName>
-    <definedName name="Heute" localSheetId="0">TODAY()</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Projektplan!$5:$7</definedName>
-    <definedName name="Projektanfang">Projektplan!$E$4</definedName>
-    <definedName name="task_end" localSheetId="0">Projektplan!$F1</definedName>
-    <definedName name="task_progress" localSheetId="0">Projektplan!$D1</definedName>
-    <definedName name="task_start" localSheetId="0">Projektplan!$E1</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Projektplan!$5:$7</definedName>
+    <definedName function="false" hidden="false" name="Anzeigewoche" vbProcedure="false">Projektplan!$E$5</definedName>
+    <definedName function="false" hidden="false" name="Projektanfang" vbProcedure="false">Projektplan!$E$4</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="Heute" vbProcedure="false">TODAY()</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="task_end" vbProcedure="false">Projektplan!$F1</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="task_progress" vbProcedure="false">Projektplan!$D1</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="task_start" vbProcedure="false">Projektplan!$E1</definedName>
   </definedNames>
-  <calcPr calcId="191028" iterateDelta="1E-4" calcCompleted="0"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -41,81 +30,81 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="76">
-  <si>
-    <t>Erstellen Sie auf diesem Arbeitsblatt einen Projektplan.
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="74">
+  <si>
+    <t xml:space="preserve">Erstellen Sie auf diesem Arbeitsblatt einen Projektplan.
 Geben Sie den Titel dieses Projekts in Zelle B1 ein. 
 Informationen zur Verwendung dieses Arbeitsblatts, einschließlich Anweisungen für die Sprachausgabe und den Verfasser dieser Arbeitsmappe, finden Sie auf dem Arbeitsblatt "Info".
 Navigieren Sie weiterhin in Spalte A abwärts, um weitere Anweisungen zu hören.</t>
   </si>
   <si>
-    <t>InvertedPendulum</t>
-  </si>
-  <si>
-    <t>Geben Sie den Firmennamen in Zelle B2 ein.</t>
+    <t xml:space="preserve">InvertedPendulum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geben Sie den Firmennamen in Zelle B2 ein.</t>
   </si>
   <si>
     <t xml:space="preserve">NwT HSG </t>
   </si>
   <si>
-    <t>Projektteam</t>
-  </si>
-  <si>
-    <t>Leonard</t>
-  </si>
-  <si>
-    <t>Attila</t>
-  </si>
-  <si>
-    <t>Geben Sie den Namen des Projektleiters in Zelle B3 ein. Geben Sie das Startdatum für das Projekt in Zelle E3 ein. Start des Projekts: Die Bezeichnung steht in Zelle C3.</t>
-  </si>
-  <si>
-    <t>Projektanfang:</t>
-  </si>
-  <si>
-    <t>Die Anzeigewoche in Zelle E4 stellt die Anfangswoche dar, die im Projektplan in Zelle I4 angezeigt werden soll. Das Startdatum des Projekts wird als Woche 1 betrachtet. Um die Anzeigewoche zu ändern, geben Sie einfach eine neue Wochennummer in Zelle E4 ein.
+    <t xml:space="preserve">Projektteam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leonard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geben Sie den Namen des Projektleiters in Zelle B3 ein. Geben Sie das Startdatum für das Projekt in Zelle E3 ein. Start des Projekts: Die Bezeichnung steht in Zelle C3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projektanfang:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Anzeigewoche in Zelle E4 stellt die Anfangswoche dar, die im Projektplan in Zelle I4 angezeigt werden soll. Das Startdatum des Projekts wird als Woche 1 betrachtet. Um die Anzeigewoche zu ändern, geben Sie einfach eine neue Wochennummer in Zelle E4 ein.
 Das Startdatum für jede Woche, beginnend mit der Anzeigewoche aus Zelle E4, beginnt in Zelle I4 und wird automatisch berechnet. In dieser Ansicht werden 8 Wochen von Zelle I4 bis Zelle BF4 dargestellt.
 Ändern Sie diese Zellen nicht.
 Anzeigewoche: Die Bezeichnung steht in Zelle C4.</t>
   </si>
   <si>
-    <t>Anzeigewoche:</t>
-  </si>
-  <si>
-    <t>Die Zellen I5 bis BL5 enthalten die Tagesnummer der Woche für die im Zellenblock oberhalb der einzelnen Datumszellen angezeigten Woche und werden automatisch berechnet.
+    <t xml:space="preserve">Anzeigewoche:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Zellen I5 bis BL5 enthalten die Tagesnummer der Woche für die im Zellenblock oberhalb der einzelnen Datumszellen angezeigten Woche und werden automatisch berechnet.
 Ändern Sie diese Zellen nicht.
 Das heutige Datum ist rot (Hex #AD3815) hervorgehoben, vom aktuellen Datum in Zeile 5 die gesamte Datumsspalte hindurch bis zum Ende des Projektplans.</t>
   </si>
   <si>
-    <t>Diese Zeile enthält Überschriften für den Projektplan, der darunter dargestellt ist. 
+    <t xml:space="preserve">Diese Zeile enthält Überschriften für den Projektplan, der darunter dargestellt ist. 
 Navigieren Sie von B6 bis BL6, um sich die Inhalte vorsprechen zu lassen. Der erste Buchstabe jedes Tags der Woche für das Datum oberhalb der Überschrift, beginnend in Zelle I6 und fortlaufend bis Zelle BL6.
 Alle Projektzeitachsendiagramme werden automatisch basierend auf den eingegebenen Start- und Enddaten mithilfe von bedingten Formaten generiert.
 Ändern Sie die Inhalte in den Zellen in Spalten nach Spalte I beginnend mit Zelle I7 nicht.</t>
   </si>
   <si>
-    <t>AUFGABE</t>
-  </si>
-  <si>
-    <t>ZUGEWIESEN
+    <t xml:space="preserve">AUFGABE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZUGEWIESEN
 AN</t>
   </si>
   <si>
-    <t>FORTSCHRITT</t>
-  </si>
-  <si>
-    <t>START</t>
-  </si>
-  <si>
-    <t>ENDE</t>
-  </si>
-  <si>
-    <t>TAGE</t>
+    <t xml:space="preserve">FORTSCHRITT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">START</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAGE</t>
   </si>
   <si>
     <t xml:space="preserve">Löschen Sie diese Zeile nicht. Diese Zeile ist ausgeblendet, um eine Formel zu schützen, die zum Hervorheben des aktuellen Tags im Projektzeitplan verwendet wird. </t>
   </si>
   <si>
-    <t>Zelle B8 enthält den Beispieltitel „Phase 1“. 
+    <t xml:space="preserve">Zelle B8 enthält den Beispieltitel „Phase 1“. 
 Geben Sie in Zelle B8 einen neuen Titel ein.
 Geben Sie in Zelle C8 einen Namen ein, der der Phase zugewiesen wird, wenn diese für Ihr Projekt zutrifft.
 Geben Sie in Zelle D8 den Fortschritt für die gesamte Phase ein, wenn diese für Ihr Projekt zutrifft.
@@ -124,7 +113,7 @@
 Um die Phase zu löschen und nur mit Aufgaben zu arbeiten, löschen Sie einfach diese Zeile.</t>
   </si>
   <si>
-    <t>Konstruktion</t>
+    <t xml:space="preserve">Konstruktion</t>
   </si>
   <si>
     <t xml:space="preserve">Zelle B9 enthält die Beispielaufgabe „Aufgabe 1“. 
@@ -136,55 +125,55 @@
 Von Zelle I9 bis Zelle BL9 wird eine Statusleiste mit einer entsprechenden Schattierung für die eingegebenen Datumsangaben in Blöcken angezeigt. </t>
   </si>
   <si>
-    <t>Bauplan erstellen</t>
-  </si>
-  <si>
-    <t>→ Extrusionszeichnung erstellen</t>
-  </si>
-  <si>
-    <t>→ Dreitafelansicht erstellen</t>
-  </si>
-  <si>
-    <t>→ Bemaßungen hinzufügen</t>
-  </si>
-  <si>
-    <t>In den Zeilen 10 bis 13 wird das Muster aus Zeile 9 wiederholt. 
+    <t xml:space="preserve">Bauplan erstellen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Extrusionszeichnung erstellen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Dreitafelansicht erstellen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Bemaßungen hinzufügen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In den Zeilen 10 bis 13 wird das Muster aus Zeile 9 wiederholt. 
 Wiederholen Sie die Anweisungen aus Zelle A9 für alle Aufgabenzeilen auf diesem Arbeitsblatt. Überschreiben Sie alle Beispieldaten.
 Ein Beispiel für eine andere Phase beginnt in Zelle A14. 
 Setzen Sie die Eingabe von Aufgaben in den Zellen A10 bis A13 fort, oder wechseln Sie zu Zelle A14, um weitere Informationen zu erhalten.</t>
   </si>
   <si>
-    <t>Strukturmodell designen</t>
-  </si>
-  <si>
-    <t>→ Untergestell</t>
-  </si>
-  <si>
-    <t>→ Obergestell</t>
-  </si>
-  <si>
-    <t>→ Platinenhalterung</t>
-  </si>
-  <si>
-    <t>→ Motorhalterung</t>
-  </si>
-  <si>
-    <t>Slidersystem entwickeln</t>
-  </si>
-  <si>
-    <t>Abhängigkeiten vorbereiten</t>
-  </si>
-  <si>
-    <t>→Motor designen</t>
-  </si>
-  <si>
-    <t>→Platine designen</t>
-  </si>
-  <si>
-    <t>Aufgabe 5</t>
-  </si>
-  <si>
-    <t>Die Zelle rechts enthält den Beispieltitel „Phase 2“. 
+    <t xml:space="preserve">Strukturmodell designen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Untergestell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Obergestell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Platinenhalterung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→ Motorhalterung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slidersystem entwickeln</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abhängigkeiten vorbereiten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→Motor designen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">→Platine designen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Komplettes Rework des gesamten Systems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Zelle rechts enthält den Beispieltitel „Phase 2“. 
 Sie können jederzeit in Spalte B eine neue Phase erstellen. In diesem Projektplan sind keine Phasen erforderlich. Um die Phase zu entfernen, löschen Sie einfach die Zeile.
 Zum Erstellen eines neuen Phasenblocks in dieser Zeile geben Sie in der Zelle rechts einen Titel ein.
 Um der Phase oben weitere Aufgaben hinzuzufügen, geben Sie über dieser Zeile eine neue Zeile ein, und tragen Sie die Aufgabendaten wie in den Anweisungen in Zelle A9 ein.
@@ -194,77 +183,83 @@
 Wiederholen Sie bei Bedarf die Anweisungen aus den Zellen A8 und A9.</t>
   </si>
   <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>PID Rechnung</t>
-  </si>
-  <si>
-    <t>Motoren einbinden</t>
-  </si>
-  <si>
-    <t>BNO055 einbinden</t>
-  </si>
-  <si>
-    <t>Code kommentieren</t>
-  </si>
-  <si>
-    <t>Code ausprobieren</t>
-  </si>
-  <si>
-    <t>Titelblock für Beispielphase</t>
-  </si>
-  <si>
-    <t>Schaltkreis</t>
-  </si>
-  <si>
-    <t>Schaltplan entwickeln</t>
-  </si>
-  <si>
-    <t>BNO055 anschließen</t>
-  </si>
-  <si>
-    <t>Motoren anschließen</t>
-  </si>
-  <si>
-    <t>Alles zusammenschließen</t>
-  </si>
-  <si>
-    <t>Vorbereitung Code/Schaltplan</t>
-  </si>
-  <si>
-    <t>Regelkreisschema</t>
-  </si>
-  <si>
-    <t>Programmablaufplan</t>
-  </si>
-  <si>
-    <t>Dies ist eine leere Zeile.</t>
-  </si>
-  <si>
-    <t>Diese Zeile kennzeichnet das Ende des Projektplans. Geben Sie in dieser Zeile NICHTS EIN. 
+    <t xml:space="preserve">Code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PID Rechnung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motoren einbinden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BNO055 einbinden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code kommentieren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code optimieren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29.03.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code ausprobieren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titelblock für Beispielphase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schaltkreis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schaltplan entwickeln</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BNO055 anschließen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motoren anschließen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alles zusammenschließen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vorbereitung Code/Schaltplan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regelkreisschema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programmablaufplan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dies ist eine leere Zeile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diese Zeile kennzeichnet das Ende des Projektplans. Geben Sie in dieser Zeile NICHTS EIN. 
 Fügen Sie ÜBER dieser Zeile neue Zeilen ein, um mit der Erstellung Ihres Projektplans fortzufahren.</t>
   </si>
   <si>
-    <t>Neue Zeilen ÜBER dieser einfügen</t>
-  </si>
-  <si>
-    <t>EINFACHES GANTT-DIAGRAMM von Vertex42.com</t>
-  </si>
-  <si>
-    <t>https://www.vertex42.com/ExcelTemplates/simple-gantt-chart.html</t>
-  </si>
-  <si>
-    <t>Über diese Vorlage</t>
-  </si>
-  <si>
-    <t>Diese Vorlage bietet eine einfache Möglichkeit, ein Gantt-Diagramm zu erstellen, um Ihr Projekt zu visualisieren und seine Nachverfolgung zu erleichtern. Geben Sie einfach Ihre Aufgaben sowie das Start- und Enddatum ein; es sind keine Formeln erforderlich. Die Balken im Gantt-Diagramm stellen die Dauer der Aufgabe dar und werden mithilfe bedingtes Formatierungen angezeigt. Fügen Sie neue Aufgaben ein, indem Sie neue Zeilen einfügen.</t>
-  </si>
-  <si>
-    <t>Leitfaden für die Sprachausgabe</t>
-  </si>
-  <si>
-    <t>Diese Arbeitsmappe enthält 2 Arbeitsblätter. 
+    <t xml:space="preserve">Neue Zeilen ÜBER dieser einfügen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EINFACHES GANTT-DIAGRAMM von Vertex42.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.vertex42.com/ExcelTemplates/simple-gantt-chart.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Über diese Vorlage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diese Vorlage bietet eine einfache Möglichkeit, ein Gantt-Diagramm zu erstellen, um Ihr Projekt zu visualisieren und seine Nachverfolgung zu erleichtern. Geben Sie einfach Ihre Aufgaben sowie das Start- und Enddatum ein; es sind keine Formeln erforderlich. Die Balken im Gantt-Diagramm stellen die Dauer der Aufgabe dar und werden mithilfe bedingtes Formatierungen angezeigt. Fügen Sie neue Aufgaben ein, indem Sie neue Zeilen einfügen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leitfaden für die Sprachausgabe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diese Arbeitsmappe enthält 2 Arbeitsblätter. 
 Arbeitszeittabelle
 Info
 Die Anweisungen für jedes Arbeitsblatt befinden sich in Spalte A ab Zelle A1 der einzelnen Arbeitsblätter. Sie sind in verborgenem Text geschrieben. Jeder Schritt führt Sie durch die Informationen in der betreffenden Zeile. Jeder nachfolgende Schritt fährt in den Zellen A2, A3 usw. fort, sofern nicht ausdrücklich anders angegeben. Beispielsweise kann der Anweisungstext etwa für den nächsten Schritt "Mit Zelle 6 fortfahren" besagen. 
@@ -272,57 +267,67 @@
 Um diese Anweisungen aus dem Arbeitsblatt zu entfernen, löschen Sie einfach Spalte A.</t>
   </si>
   <si>
-    <t>Weitere Hilfe</t>
-  </si>
-  <si>
-    <t>Klicken Sie auf den Link unten, um zu vertex42.com zu gehen und mehr über die Verwendung dieser Vorlage zu erfahren, z. B. wie Tage und Arbeitstage berechnet werden, wie Aufgabenabhängigkeiten erstellt werden, wie die Farben der Balken geändert werden, wie eine Bildlaufleiste hinzugefügt wird, um die Anzeigewoche einfacher zu ändern, wie der in dem Diagramm angezeigte Datumsbereich geändert wird usw.</t>
-  </si>
-  <si>
-    <t>Verwenden des einfachen Gantt-Diagramms</t>
-  </si>
-  <si>
-    <t>Weitere Projektmanagementvorlagen</t>
-  </si>
-  <si>
-    <t>Rufen Sie Vertex42.com auf, um weitere Projektmanagementvorlagen herunterzuladen, einschließlich unterschiedlicher Typen von Projektplänen, Gantt-Diagramme, Aufgabenlisten usw.</t>
-  </si>
-  <si>
-    <t>Projektmanagementvorlagen</t>
-  </si>
-  <si>
-    <t>Informationen zu Vertex42</t>
-  </si>
-  <si>
-    <t>Vertex42.com bietet mehr als 300 professionell entworfene Tabellenkalkulationsvorlagen für die Nutzung im Geschäft, zu Hause und in Bildungseinrichtungen – die meisten können Sie kostenlos herunterladen. Die Sammlung beinhaltet eine Vielzahl von Kalendern, Planern und Zeitplänen sowie Tabellen für die private Finanzkalkulation zur Erstellung von Budgets, Reduzierung von Belastungen und Amortisation von Darlehen.</t>
-  </si>
-  <si>
-    <t>Unternehmen werden bei Rechnungen, Arbeitszeittabellen, Bestandstrackern, Geschäftsberichten und Vorlagen für die Projektplanung fündig. Lehrer und Schüler finden Ressourcen wie Stundenpläne, Klassenbücher und Teilnahmebögen. Organisieren Sie Ihr Familienleben mit Speiseplänen, Checklisten und Übungsprotokollen. Jede Vorlage wurde gründlich recherchiert, verfeinert und im Lauf der Zeit anhand des Feedbacks von Tausenden von Benutzern verbessert.</t>
-  </si>
-  <si>
-    <t>Code optimieren</t>
-  </si>
-  <si>
-    <t>29.03.2026</t>
+    <t xml:space="preserve">Weitere Hilfe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klicken Sie auf den Link unten, um zu vertex42.com zu gehen und mehr über die Verwendung dieser Vorlage zu erfahren, z. B. wie Tage und Arbeitstage berechnet werden, wie Aufgabenabhängigkeiten erstellt werden, wie die Farben der Balken geändert werden, wie eine Bildlaufleiste hinzugefügt wird, um die Anzeigewoche einfacher zu ändern, wie der in dem Diagramm angezeigte Datumsbereich geändert wird usw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verwenden des einfachen Gantt-Diagramms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weitere Projektmanagementvorlagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rufen Sie Vertex42.com auf, um weitere Projektmanagementvorlagen herunterzuladen, einschließlich unterschiedlicher Typen von Projektplänen, Gantt-Diagramme, Aufgabenlisten usw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projektmanagementvorlagen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informationen zu Vertex42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertex42.com bietet mehr als 300 professionell entworfene Tabellenkalkulationsvorlagen für die Nutzung im Geschäft, zu Hause und in Bildungseinrichtungen – die meisten können Sie kostenlos herunterladen. Die Sammlung beinhaltet eine Vielzahl von Kalendern, Planern und Zeitplänen sowie Tabellen für die private Finanzkalkulation zur Erstellung von Budgets, Reduzierung von Belastungen und Amortisation von Darlehen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unternehmen werden bei Rechnungen, Arbeitszeittabellen, Bestandstrackern, Geschäftsberichten und Vorlagen für die Projektplanung fündig. Lehrer und Schüler finden Ressourcen wie Stundenpläne, Klassenbücher und Teilnahmebögen. Organisieren Sie Ihr Familienleben mit Speiseplänen, Checklisten und Übungsprotokollen. Jede Vorlage wurde gründlich recherchiert, verfeinert und im Lauf der Zeit anhand des Feedbacks von Tausenden von Benutzern verbessert.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="d/m/yy;@"/>
-    <numFmt numFmtId="165" formatCode="ddd&quot;, &quot;d/m/yyyy"/>
-    <numFmt numFmtId="166" formatCode="d/\ mmm\ yyyy"/>
-    <numFmt numFmtId="167" formatCode="d"/>
-    <numFmt numFmtId="168" formatCode="0\ %"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="6">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="d/m/yy;@"/>
+    <numFmt numFmtId="166" formatCode="ddd&quot;, &quot;d/m/yyyy"/>
+    <numFmt numFmtId="167" formatCode="d/\ mmm\ yyyy"/>
+    <numFmt numFmtId="168" formatCode="d"/>
+    <numFmt numFmtId="169" formatCode="0\ %"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -332,17 +337,17 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="22"/>
-      <color theme="1" tint="0.3498947111423078"/>
+      <color theme="1" tint="0.3498"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="20"/>
-      <color theme="4" tint="-0.249977111117893"/>
+      <color theme="4" tint="-0.25"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -354,7 +359,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
@@ -369,7 +374,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <u/>
+      <u val="single"/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
@@ -390,7 +395,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="9"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -405,7 +410,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -419,13 +424,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <i/>
+      <i val="true"/>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -434,36 +433,36 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1" tint="0.49989318521683401"/>
+      <color theme="1" tint="0.4998"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
-      <color theme="1" tint="0.49989318521683401"/>
+      <color theme="1" tint="0.4998"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
-      <color theme="1" tint="0.49989318521683401"/>
+      <color theme="1" tint="0.4998"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="12"/>
-      <color theme="1" tint="0.3498947111423078"/>
+      <color theme="1" tint="0.3498"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -478,15 +477,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1" tint="0.49989318521683401"/>
+      <color theme="1" tint="0.4998"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="16"/>
-      <color theme="4" tint="-0.249977111117893"/>
+      <color theme="4" tint="-0.25"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -504,13 +503,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="17">
     <fill>
@@ -521,7 +513,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79989013336588644"/>
+        <fgColor theme="5" tint="0.7998"/>
         <bgColor rgb="FFE6E0EC"/>
       </patternFill>
     </fill>
@@ -533,37 +525,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79989013336588644"/>
+        <fgColor theme="8" tint="0.7998"/>
         <bgColor rgb="FFDAEEF3"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.15"/>
         <bgColor rgb="FFE6E0EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="1" tint="0.3498947111423078"/>
+        <fgColor theme="1" tint="0.3498"/>
         <bgColor rgb="FF376092"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59987182226020086"/>
+        <fgColor theme="4" tint="0.5998"/>
         <bgColor rgb="FFCCC1DA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79989013336588644"/>
+        <fgColor theme="4" tint="0.7998"/>
         <bgColor rgb="FFDBEEF4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59987182226020086"/>
+        <fgColor theme="5" tint="0.5998"/>
         <bgColor rgb="FFCCC1DA"/>
       </patternFill>
     </fill>
@@ -581,470 +573,636 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59987182226020086"/>
+        <fgColor theme="6" tint="0.5998"/>
         <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79989013336588644"/>
+        <fgColor theme="6" tint="0.7998"/>
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59987182226020086"/>
+        <fgColor theme="7" tint="0.5998"/>
         <bgColor rgb="FFB9CDE5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79989013336588644"/>
+        <fgColor theme="7" tint="0.7998"/>
         <bgColor rgb="FFDCE6F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <fgColor theme="0" tint="-0.05"/>
         <bgColor rgb="FFEBF1DE"/>
       </patternFill>
     </fill>
   </fills>
   <borders count="10">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top style="medium">
-        <color theme="0" tint="-0.14999847407452621"/>
+        <color theme="0" tint="-0.15"/>
       </top>
       <bottom style="medium">
-        <color theme="0" tint="-0.14999847407452621"/>
+        <color theme="0" tint="-0.15"/>
       </bottom>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </left>
       <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </right>
       <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </top>
       <bottom style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </bottom>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </left>
       <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </right>
       <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </bottom>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </left>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </left>
       <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
+        <color theme="0" tint="-0.35"/>
       </right>
       <top/>
       <bottom style="medium">
-        <color theme="0" tint="-0.14999847407452621"/>
+        <color theme="0" tint="-0.15"/>
       </bottom>
       <diagonal/>
     </border>
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
+        <color theme="0" tint="-0.15"/>
       </left>
       <right style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
+        <color theme="0" tint="-0.15"/>
       </right>
       <top style="medium">
-        <color theme="0" tint="-0.14999847407452621"/>
+        <color theme="0" tint="-0.15"/>
       </top>
       <bottom style="medium">
-        <color theme="0" tint="-0.14999847407452621"/>
+        <color theme="0" tint="-0.15"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="12">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="168" fontId="26" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="0" borderId="2">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyProtection="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyProtection="0">
-      <alignment horizontal="right" indent="1"/>
+  <cellStyleXfs count="30">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="100">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="11" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="9" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="10" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="8" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="9" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="12" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="13" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="13" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="14" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="14" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="15" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="15" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="13" fillId="16" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
+  <cellXfs count="97">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="26" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="27" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="28" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="29" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="2" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="5" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="12" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="7" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="8" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="9" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="2" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="12" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="13" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="13" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="14" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="14" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="14" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="15" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="15" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="23" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="16" borderId="1" xfId="19" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="16" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="12">
-    <cellStyle name="Aufgabe" xfId="3" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Datum" xfId="4" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Excel Built-in Heading 1" xfId="9" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="Excel Built-in Heading 2" xfId="10" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="Excel Built-in Heading 3" xfId="11" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="Excel Built-in Title" xfId="8" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="Name" xfId="5" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
+  <cellStyles count="16">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
-    <cellStyle name="Projektanfang" xfId="6" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="zAusgeblText" xfId="7" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Aufgabe" xfId="21"/>
+    <cellStyle name="Datum" xfId="22"/>
+    <cellStyle name="Name" xfId="23"/>
+    <cellStyle name="Projektanfang" xfId="24"/>
+    <cellStyle name="zAusgeblText" xfId="25"/>
+    <cellStyle name="Excel Built-in Title" xfId="26"/>
+    <cellStyle name="Excel Built-in Heading 1" xfId="27"/>
+    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
+    <cellStyle name="Excel Built-in Heading 2" xfId="28"/>
+    <cellStyle name="Excel Built-in Heading 3" xfId="29"/>
   </cellStyles>
   <dxfs count="9">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFEBF1DE"/>
+          <bgColor theme="8" tint="-0.25"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6" tint="-0.25"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.25"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1058,21 +1216,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="-0.249977111117893"/>
+          <bgColor rgb="FFEBF1DE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1086,25 +1230,26 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="0" tint="-0.35"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="false" diagonalDown="false">
         <left/>
         <right/>
         <top/>
         <bottom/>
+        <diagonal/>
       </border>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.34998626667073579"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <border diagonalUp="false" diagonalDown="false">
         <left style="thin">
           <color rgb="FFC00000"/>
         </left>
@@ -1113,10 +1258,10 @@
         </right>
         <top/>
         <bottom/>
+        <diagonal/>
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1175,29 +1320,13 @@
       <rgbColor rgb="FF7030A0"/>
       <rgbColor rgb="FF376092"/>
       <rgbColor rgb="FF1D2129"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -1207,30 +1336,25 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1903320</xdr:colOff>
+      <xdr:colOff>1902960</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>522360</xdr:rowOff>
+      <xdr:rowOff>522000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Bild 1" descr="Vertex42-Logo">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
-            </a:ext>
-          </a:extLst>
+        <xdr:cNvPr id="1" name="Bild 1" descr="Vertex42-Logo">
+          <a:hlinkClick r:id="rId1"/>
         </xdr:cNvPr>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:blip r:embed="rId2"/>
         <a:stretch/>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="95400"/>
-          <a:ext cx="1903320" cy="426960"/>
+          <a:ext cx="1902960" cy="426600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1247,7 +1371,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2007-2010">
       <a:dk1>
@@ -1289,12 +1413,12 @@
     </a:clrScheme>
     <a:fontScheme name="Calibri">
       <a:majorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -1326,7 +1450,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1350,7 +1474,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1410,179 +1534,177 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:BR1048576"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:BL1048576"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="30" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="2.6875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="32.28515625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="11.703125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="10.76171875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="10.4921875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="10.4921875" style="5" customWidth="1"/>
-    <col min="7" max="7" width="2.6875" style="5" customWidth="1"/>
-    <col min="8" max="8" width="6.1875" style="5" hidden="1" customWidth="1"/>
-    <col min="9" max="64" width="2.41796875" style="5" customWidth="1"/>
-    <col min="69" max="70" width="10.22265625" style="5" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="43.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="11.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="10.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="10.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="2.69"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="2" width="6.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="9" style="2" width="2.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="69" style="2" width="10.22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="12"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="13"/>
-    </row>
-    <row r="2" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="9"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="10"/>
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="15"/>
-    </row>
-    <row r="3" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="16" t="s">
+      <c r="I2" s="12"/>
+    </row>
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="18" t="s">
+      <c r="D3" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="19"/>
-      <c r="I3" s="15"/>
-    </row>
-    <row r="4" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="E3" s="16"/>
+      <c r="I3" s="12"/>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="2">
+      <c r="D4" s="17"/>
+      <c r="E4" s="18" t="n">
         <v>46008</v>
       </c>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
+      <c r="F4" s="18"/>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="20">
+      <c r="D5" s="17"/>
+      <c r="E5" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="I5" s="1">
-        <f>I6</f>
+      <c r="I5" s="20" t="n">
+        <f aca="false">I6</f>
         <v>46069</v>
       </c>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1">
-        <f>P6</f>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20" t="n">
+        <f aca="false">P6</f>
         <v>46076</v>
       </c>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="S5" s="1"/>
-      <c r="T5" s="1"/>
-      <c r="U5" s="1"/>
-      <c r="V5" s="1"/>
-      <c r="W5" s="1">
-        <f>W6</f>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="20" t="n">
+        <f aca="false">W6</f>
         <v>46083</v>
       </c>
-      <c r="X5" s="1"/>
-      <c r="Y5" s="1"/>
-      <c r="Z5" s="1"/>
-      <c r="AA5" s="1"/>
-      <c r="AB5" s="1"/>
-      <c r="AC5" s="1"/>
-      <c r="AD5" s="1">
-        <f>AD6</f>
+      <c r="X5" s="20"/>
+      <c r="Y5" s="20"/>
+      <c r="Z5" s="20"/>
+      <c r="AA5" s="20"/>
+      <c r="AB5" s="20"/>
+      <c r="AC5" s="20"/>
+      <c r="AD5" s="20" t="n">
+        <f aca="false">AD6</f>
         <v>46090</v>
       </c>
-      <c r="AE5" s="1"/>
-      <c r="AF5" s="1"/>
-      <c r="AG5" s="1"/>
-      <c r="AH5" s="1"/>
-      <c r="AI5" s="1"/>
-      <c r="AJ5" s="1"/>
-      <c r="AK5" s="1">
-        <f>AK6</f>
+      <c r="AE5" s="20"/>
+      <c r="AF5" s="20"/>
+      <c r="AG5" s="20"/>
+      <c r="AH5" s="20"/>
+      <c r="AI5" s="20"/>
+      <c r="AJ5" s="20"/>
+      <c r="AK5" s="20" t="n">
+        <f aca="false">AK6</f>
         <v>46097</v>
       </c>
-      <c r="AL5" s="1"/>
-      <c r="AM5" s="1"/>
-      <c r="AN5" s="1"/>
-      <c r="AO5" s="1"/>
-      <c r="AP5" s="1"/>
-      <c r="AQ5" s="1"/>
-      <c r="AR5" s="1">
-        <f>AR6</f>
+      <c r="AL5" s="20"/>
+      <c r="AM5" s="20"/>
+      <c r="AN5" s="20"/>
+      <c r="AO5" s="20"/>
+      <c r="AP5" s="20"/>
+      <c r="AQ5" s="20"/>
+      <c r="AR5" s="20" t="n">
+        <f aca="false">AR6</f>
         <v>46104</v>
       </c>
-      <c r="AS5" s="1"/>
-      <c r="AT5" s="1"/>
-      <c r="AU5" s="1"/>
-      <c r="AV5" s="1"/>
-      <c r="AW5" s="1"/>
-      <c r="AX5" s="1"/>
-      <c r="AY5" s="1">
-        <f>AY6</f>
+      <c r="AS5" s="20"/>
+      <c r="AT5" s="20"/>
+      <c r="AU5" s="20"/>
+      <c r="AV5" s="20"/>
+      <c r="AW5" s="20"/>
+      <c r="AX5" s="20"/>
+      <c r="AY5" s="20" t="n">
+        <f aca="false">AY6</f>
         <v>46111</v>
       </c>
-      <c r="AZ5" s="1"/>
-      <c r="BA5" s="1"/>
-      <c r="BB5" s="1"/>
-      <c r="BC5" s="1"/>
-      <c r="BD5" s="1"/>
-      <c r="BE5" s="1"/>
-      <c r="BF5" s="1">
-        <f>BF6</f>
+      <c r="AZ5" s="20"/>
+      <c r="BA5" s="20"/>
+      <c r="BB5" s="20"/>
+      <c r="BC5" s="20"/>
+      <c r="BD5" s="20"/>
+      <c r="BE5" s="20"/>
+      <c r="BF5" s="20" t="n">
+        <f aca="false">BF6</f>
         <v>46118</v>
       </c>
-      <c r="BG5" s="1"/>
-      <c r="BH5" s="1"/>
-      <c r="BI5" s="1"/>
-      <c r="BJ5" s="1"/>
-      <c r="BK5" s="1"/>
-      <c r="BL5" s="1"/>
-    </row>
-    <row r="6" spans="1:64" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="7" t="s">
+      <c r="BG5" s="20"/>
+      <c r="BH5" s="20"/>
+      <c r="BI5" s="20"/>
+      <c r="BJ5" s="20"/>
+      <c r="BK5" s="20"/>
+      <c r="BL5" s="20"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="21"/>
@@ -1591,233 +1713,233 @@
       <c r="E6" s="21"/>
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
-      <c r="I6" s="22">
-        <f>Projektanfang-WEEKDAY(Projektanfang,1)+2+7*(Anzeigewoche-1)</f>
+      <c r="I6" s="22" t="n">
+        <f aca="false">Projektanfang-WEEKDAY(Projektanfang,1)+2+7*(Anzeigewoche-1)</f>
         <v>46069</v>
       </c>
-      <c r="J6" s="23">
-        <f>I6+1</f>
+      <c r="J6" s="23" t="n">
+        <f aca="false">I6+1</f>
         <v>46070</v>
       </c>
-      <c r="K6" s="23">
-        <f>J6+1</f>
+      <c r="K6" s="23" t="n">
+        <f aca="false">J6+1</f>
         <v>46071</v>
       </c>
-      <c r="L6" s="23">
-        <f>K6+1</f>
+      <c r="L6" s="23" t="n">
+        <f aca="false">K6+1</f>
         <v>46072</v>
       </c>
-      <c r="M6" s="23">
-        <f>L6+1</f>
+      <c r="M6" s="23" t="n">
+        <f aca="false">L6+1</f>
         <v>46073</v>
       </c>
-      <c r="N6" s="23">
-        <f>M6+1</f>
+      <c r="N6" s="23" t="n">
+        <f aca="false">M6+1</f>
         <v>46074</v>
       </c>
-      <c r="O6" s="24">
-        <f>N6+1</f>
+      <c r="O6" s="24" t="n">
+        <f aca="false">N6+1</f>
         <v>46075</v>
       </c>
-      <c r="P6" s="22">
-        <f>O6+1</f>
+      <c r="P6" s="22" t="n">
+        <f aca="false">O6+1</f>
         <v>46076</v>
       </c>
-      <c r="Q6" s="23">
-        <f>P6+1</f>
+      <c r="Q6" s="23" t="n">
+        <f aca="false">P6+1</f>
         <v>46077</v>
       </c>
-      <c r="R6" s="23">
-        <f>Q6+1</f>
+      <c r="R6" s="23" t="n">
+        <f aca="false">Q6+1</f>
         <v>46078</v>
       </c>
-      <c r="S6" s="23">
-        <f>R6+1</f>
+      <c r="S6" s="23" t="n">
+        <f aca="false">R6+1</f>
         <v>46079</v>
       </c>
-      <c r="T6" s="23">
-        <f>S6+1</f>
+      <c r="T6" s="23" t="n">
+        <f aca="false">S6+1</f>
         <v>46080</v>
       </c>
-      <c r="U6" s="23">
-        <f>T6+1</f>
+      <c r="U6" s="23" t="n">
+        <f aca="false">T6+1</f>
         <v>46081</v>
       </c>
-      <c r="V6" s="24">
-        <f>U6+1</f>
+      <c r="V6" s="24" t="n">
+        <f aca="false">U6+1</f>
         <v>46082</v>
       </c>
-      <c r="W6" s="22">
-        <f>V6+1</f>
+      <c r="W6" s="22" t="n">
+        <f aca="false">V6+1</f>
         <v>46083</v>
       </c>
-      <c r="X6" s="23">
-        <f>W6+1</f>
+      <c r="X6" s="23" t="n">
+        <f aca="false">W6+1</f>
         <v>46084</v>
       </c>
-      <c r="Y6" s="23">
-        <f>X6+1</f>
+      <c r="Y6" s="23" t="n">
+        <f aca="false">X6+1</f>
         <v>46085</v>
       </c>
-      <c r="Z6" s="23">
-        <f>Y6+1</f>
+      <c r="Z6" s="23" t="n">
+        <f aca="false">Y6+1</f>
         <v>46086</v>
       </c>
-      <c r="AA6" s="23">
-        <f>Z6+1</f>
+      <c r="AA6" s="23" t="n">
+        <f aca="false">Z6+1</f>
         <v>46087</v>
       </c>
-      <c r="AB6" s="23">
-        <f>AA6+1</f>
+      <c r="AB6" s="23" t="n">
+        <f aca="false">AA6+1</f>
         <v>46088</v>
       </c>
-      <c r="AC6" s="24">
-        <f>AB6+1</f>
+      <c r="AC6" s="24" t="n">
+        <f aca="false">AB6+1</f>
         <v>46089</v>
       </c>
-      <c r="AD6" s="22">
-        <f>AC6+1</f>
+      <c r="AD6" s="22" t="n">
+        <f aca="false">AC6+1</f>
         <v>46090</v>
       </c>
-      <c r="AE6" s="23">
-        <f>AD6+1</f>
+      <c r="AE6" s="23" t="n">
+        <f aca="false">AD6+1</f>
         <v>46091</v>
       </c>
-      <c r="AF6" s="23">
-        <f>AE6+1</f>
+      <c r="AF6" s="23" t="n">
+        <f aca="false">AE6+1</f>
         <v>46092</v>
       </c>
-      <c r="AG6" s="23">
-        <f>AF6+1</f>
+      <c r="AG6" s="23" t="n">
+        <f aca="false">AF6+1</f>
         <v>46093</v>
       </c>
-      <c r="AH6" s="23">
-        <f>AG6+1</f>
+      <c r="AH6" s="23" t="n">
+        <f aca="false">AG6+1</f>
         <v>46094</v>
       </c>
-      <c r="AI6" s="23">
-        <f>AH6+1</f>
+      <c r="AI6" s="23" t="n">
+        <f aca="false">AH6+1</f>
         <v>46095</v>
       </c>
-      <c r="AJ6" s="24">
-        <f>AI6+1</f>
+      <c r="AJ6" s="24" t="n">
+        <f aca="false">AI6+1</f>
         <v>46096</v>
       </c>
-      <c r="AK6" s="22">
-        <f>AJ6+1</f>
+      <c r="AK6" s="22" t="n">
+        <f aca="false">AJ6+1</f>
         <v>46097</v>
       </c>
-      <c r="AL6" s="23">
-        <f>AK6+1</f>
+      <c r="AL6" s="23" t="n">
+        <f aca="false">AK6+1</f>
         <v>46098</v>
       </c>
-      <c r="AM6" s="23">
-        <f>AL6+1</f>
+      <c r="AM6" s="23" t="n">
+        <f aca="false">AL6+1</f>
         <v>46099</v>
       </c>
-      <c r="AN6" s="23">
-        <f>AM6+1</f>
+      <c r="AN6" s="23" t="n">
+        <f aca="false">AM6+1</f>
         <v>46100</v>
       </c>
-      <c r="AO6" s="23">
-        <f>AN6+1</f>
+      <c r="AO6" s="23" t="n">
+        <f aca="false">AN6+1</f>
         <v>46101</v>
       </c>
-      <c r="AP6" s="23">
-        <f>AO6+1</f>
+      <c r="AP6" s="23" t="n">
+        <f aca="false">AO6+1</f>
         <v>46102</v>
       </c>
-      <c r="AQ6" s="24">
-        <f>AP6+1</f>
+      <c r="AQ6" s="24" t="n">
+        <f aca="false">AP6+1</f>
         <v>46103</v>
       </c>
-      <c r="AR6" s="22">
-        <f>AQ6+1</f>
+      <c r="AR6" s="22" t="n">
+        <f aca="false">AQ6+1</f>
         <v>46104</v>
       </c>
-      <c r="AS6" s="23">
-        <f>AR6+1</f>
+      <c r="AS6" s="23" t="n">
+        <f aca="false">AR6+1</f>
         <v>46105</v>
       </c>
-      <c r="AT6" s="23">
-        <f>AS6+1</f>
+      <c r="AT6" s="23" t="n">
+        <f aca="false">AS6+1</f>
         <v>46106</v>
       </c>
-      <c r="AU6" s="23">
-        <f>AT6+1</f>
+      <c r="AU6" s="23" t="n">
+        <f aca="false">AT6+1</f>
         <v>46107</v>
       </c>
-      <c r="AV6" s="23">
-        <f>AU6+1</f>
+      <c r="AV6" s="23" t="n">
+        <f aca="false">AU6+1</f>
         <v>46108</v>
       </c>
-      <c r="AW6" s="23">
-        <f>AV6+1</f>
+      <c r="AW6" s="23" t="n">
+        <f aca="false">AV6+1</f>
         <v>46109</v>
       </c>
-      <c r="AX6" s="24">
-        <f>AW6+1</f>
+      <c r="AX6" s="24" t="n">
+        <f aca="false">AW6+1</f>
         <v>46110</v>
       </c>
-      <c r="AY6" s="22">
-        <f>AX6+1</f>
+      <c r="AY6" s="22" t="n">
+        <f aca="false">AX6+1</f>
         <v>46111</v>
       </c>
-      <c r="AZ6" s="23">
-        <f>AY6+1</f>
+      <c r="AZ6" s="23" t="n">
+        <f aca="false">AY6+1</f>
         <v>46112</v>
       </c>
-      <c r="BA6" s="23">
-        <f>AZ6+1</f>
+      <c r="BA6" s="23" t="n">
+        <f aca="false">AZ6+1</f>
         <v>46113</v>
       </c>
-      <c r="BB6" s="23">
-        <f>BA6+1</f>
+      <c r="BB6" s="23" t="n">
+        <f aca="false">BA6+1</f>
         <v>46114</v>
       </c>
-      <c r="BC6" s="23">
-        <f>BB6+1</f>
+      <c r="BC6" s="23" t="n">
+        <f aca="false">BB6+1</f>
         <v>46115</v>
       </c>
-      <c r="BD6" s="23">
-        <f>BC6+1</f>
+      <c r="BD6" s="23" t="n">
+        <f aca="false">BC6+1</f>
         <v>46116</v>
       </c>
-      <c r="BE6" s="24">
-        <f>BD6+1</f>
+      <c r="BE6" s="24" t="n">
+        <f aca="false">BD6+1</f>
         <v>46117</v>
       </c>
-      <c r="BF6" s="22">
-        <f>BE6+1</f>
+      <c r="BF6" s="22" t="n">
+        <f aca="false">BE6+1</f>
         <v>46118</v>
       </c>
-      <c r="BG6" s="23">
-        <f>BF6+1</f>
+      <c r="BG6" s="23" t="n">
+        <f aca="false">BF6+1</f>
         <v>46119</v>
       </c>
-      <c r="BH6" s="23">
-        <f>BG6+1</f>
+      <c r="BH6" s="23" t="n">
+        <f aca="false">BG6+1</f>
         <v>46120</v>
       </c>
-      <c r="BI6" s="23">
-        <f>BH6+1</f>
+      <c r="BI6" s="23" t="n">
+        <f aca="false">BH6+1</f>
         <v>46121</v>
       </c>
-      <c r="BJ6" s="23">
-        <f>BI6+1</f>
+      <c r="BJ6" s="23" t="n">
+        <f aca="false">BI6+1</f>
         <v>46122</v>
       </c>
-      <c r="BK6" s="23">
-        <f>BJ6+1</f>
+      <c r="BK6" s="23" t="n">
+        <f aca="false">BJ6+1</f>
         <v>46123</v>
       </c>
-      <c r="BL6" s="24">
-        <f>BK6+1</f>
+      <c r="BL6" s="24" t="n">
+        <f aca="false">BK6+1</f>
         <v>46124</v>
       </c>
     </row>
-    <row r="7" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="7" t="s">
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="25" t="s">
@@ -1840,237 +1962,237 @@
         <v>18</v>
       </c>
       <c r="I7" s="27" t="str">
-        <f>LEFT(TEXT(I6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(I6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="J7" s="27" t="str">
-        <f>LEFT(TEXT(J6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(J6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="K7" s="27" t="str">
-        <f>LEFT(TEXT(K6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(K6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="L7" s="27" t="str">
-        <f>LEFT(TEXT(L6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(L6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="M7" s="27" t="str">
-        <f>LEFT(TEXT(M6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(M6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="N7" s="27" t="str">
-        <f>LEFT(TEXT(N6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(N6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="O7" s="27" t="str">
-        <f>LEFT(TEXT(O6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(O6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="P7" s="27" t="str">
-        <f>LEFT(TEXT(P6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(P6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="Q7" s="27" t="str">
-        <f>LEFT(TEXT(Q6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(Q6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="R7" s="27" t="str">
-        <f>LEFT(TEXT(R6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(R6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="S7" s="27" t="str">
-        <f>LEFT(TEXT(S6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(S6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="T7" s="27" t="str">
-        <f>LEFT(TEXT(T6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(T6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="U7" s="27" t="str">
-        <f>LEFT(TEXT(U6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(U6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="V7" s="27" t="str">
-        <f>LEFT(TEXT(V6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(V6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="W7" s="27" t="str">
-        <f>LEFT(TEXT(W6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(W6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="X7" s="27" t="str">
-        <f>LEFT(TEXT(X6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(X6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="Y7" s="27" t="str">
-        <f>LEFT(TEXT(Y6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(Y6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="Z7" s="27" t="str">
-        <f>LEFT(TEXT(Z6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(Z6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="AA7" s="27" t="str">
-        <f>LEFT(TEXT(AA6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AA6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="AB7" s="27" t="str">
-        <f>LEFT(TEXT(AB6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AB6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AC7" s="27" t="str">
-        <f>LEFT(TEXT(AC6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AC6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AD7" s="27" t="str">
-        <f>LEFT(TEXT(AD6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AD6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="AE7" s="27" t="str">
-        <f>LEFT(TEXT(AE6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AE6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="AF7" s="27" t="str">
-        <f>LEFT(TEXT(AF6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AF6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="AG7" s="27" t="str">
-        <f>LEFT(TEXT(AG6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AG6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="AH7" s="27" t="str">
-        <f>LEFT(TEXT(AH6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AH6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="AI7" s="27" t="str">
-        <f>LEFT(TEXT(AI6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AI6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AJ7" s="27" t="str">
-        <f>LEFT(TEXT(AJ6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AJ6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AK7" s="27" t="str">
-        <f>LEFT(TEXT(AK6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AK6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="AL7" s="27" t="str">
-        <f>LEFT(TEXT(AL6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AL6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="AM7" s="27" t="str">
-        <f>LEFT(TEXT(AM6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AM6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="AN7" s="27" t="str">
-        <f>LEFT(TEXT(AN6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AN6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="AO7" s="27" t="str">
-        <f>LEFT(TEXT(AO6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AO6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="AP7" s="27" t="str">
-        <f>LEFT(TEXT(AP6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AP6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AQ7" s="27" t="str">
-        <f>LEFT(TEXT(AQ6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AQ6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AR7" s="27" t="str">
-        <f>LEFT(TEXT(AR6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AR6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="AS7" s="27" t="str">
-        <f>LEFT(TEXT(AS6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AS6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="AT7" s="27" t="str">
-        <f>LEFT(TEXT(AT6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AT6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="AU7" s="27" t="str">
-        <f>LEFT(TEXT(AU6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AU6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="AV7" s="27" t="str">
-        <f>LEFT(TEXT(AV6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AV6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="AW7" s="27" t="str">
-        <f>LEFT(TEXT(AW6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AW6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AX7" s="27" t="str">
-        <f>LEFT(TEXT(AX6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AX6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="AY7" s="27" t="str">
-        <f>LEFT(TEXT(AY6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AY6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="AZ7" s="27" t="str">
-        <f>LEFT(TEXT(AZ6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(AZ6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="BA7" s="27" t="str">
-        <f>LEFT(TEXT(BA6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BA6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="BB7" s="27" t="str">
-        <f>LEFT(TEXT(BB6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BB6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="BC7" s="27" t="str">
-        <f>LEFT(TEXT(BC6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BC6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="BD7" s="27" t="str">
-        <f>LEFT(TEXT(BD6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BD6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="BE7" s="27" t="str">
-        <f>LEFT(TEXT(BE6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BE6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="BF7" s="27" t="str">
-        <f>LEFT(TEXT(BF6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BF6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="BG7" s="27" t="str">
-        <f>LEFT(TEXT(BG6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BG6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="BH7" s="27" t="str">
-        <f>LEFT(TEXT(BH6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BH6,"TTTT"),1)</f>
+        <v>M</v>
       </c>
       <c r="BI7" s="27" t="str">
-        <f>LEFT(TEXT(BI6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BI6,"TTTT"),1)</f>
+        <v>D</v>
       </c>
       <c r="BJ7" s="27" t="str">
-        <f>LEFT(TEXT(BJ6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BJ6,"TTTT"),1)</f>
+        <v>F</v>
       </c>
       <c r="BK7" s="27" t="str">
-        <f>LEFT(TEXT(BK6,"TTTT"),1)</f>
-        <v>T</v>
+        <f aca="false">LEFT(TEXT(BK6,"TTTT"),1)</f>
+        <v>S</v>
       </c>
       <c r="BL7" s="27" t="str">
-        <f>LEFT(TEXT(BL6,"TTTT"),1)</f>
-        <v>T</v>
-      </c>
-    </row>
-    <row r="8" spans="1:64" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+        <f aca="false">LEFT(TEXT(BL6,"TTTT"),1)</f>
+        <v>S</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="28"/>
-      <c r="H8" s="5" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H8" s="2" t="str">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I8" s="29"/>
@@ -2130,8 +2252,8 @@
       <c r="BK8" s="29"/>
       <c r="BL8" s="29"/>
     </row>
-    <row r="9" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
+    <row r="9" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
         <v>20</v>
       </c>
       <c r="B9" s="30" t="s">
@@ -2140,13 +2262,19 @@
       <c r="C9" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="32"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34"/>
+      <c r="D9" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <v>46029</v>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>46181</v>
+      </c>
       <c r="G9" s="35"/>
-      <c r="H9" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v/>
+      <c r="H9" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>153</v>
       </c>
       <c r="I9" s="29"/>
       <c r="J9" s="29"/>
@@ -2205,8 +2333,8 @@
       <c r="BK9" s="29"/>
       <c r="BL9" s="29"/>
     </row>
-    <row r="10" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="7" t="s">
+    <row r="10" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>22</v>
       </c>
       <c r="B10" s="37" t="s">
@@ -2215,17 +2343,19 @@
       <c r="C10" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="39">
-        <v>0.4</v>
-      </c>
-      <c r="E10" s="40">
+      <c r="D10" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="40" t="n">
         <v>46106</v>
       </c>
-      <c r="F10" s="40"/>
+      <c r="F10" s="40" t="n">
+        <v>46181</v>
+      </c>
       <c r="G10" s="35"/>
-      <c r="H10" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v/>
+      <c r="H10" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>76</v>
       </c>
       <c r="I10" s="29"/>
       <c r="J10" s="29"/>
@@ -2284,21 +2414,23 @@
       <c r="BK10" s="29"/>
       <c r="BL10" s="29"/>
     </row>
-    <row r="11" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="7"/>
+    <row r="11" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4"/>
       <c r="B11" s="37" t="s">
         <v>24</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D11" s="39">
-        <v>0</v>
-      </c>
-      <c r="E11" s="40">
+      <c r="D11" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="40" t="n">
         <v>46106</v>
       </c>
-      <c r="F11" s="40"/>
+      <c r="F11" s="40" t="n">
+        <v>46181</v>
+      </c>
       <c r="G11" s="35"/>
       <c r="H11" s="35"/>
       <c r="I11" s="29"/>
@@ -2358,21 +2490,23 @@
       <c r="BK11" s="29"/>
       <c r="BL11" s="29"/>
     </row>
-    <row r="12" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7"/>
+    <row r="12" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4"/>
       <c r="B12" s="37" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="39">
-        <v>0.6</v>
-      </c>
-      <c r="E12" s="40">
+      <c r="D12" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="40" t="n">
         <v>46106</v>
       </c>
-      <c r="F12" s="40"/>
+      <c r="F12" s="40" t="n">
+        <v>46106</v>
+      </c>
       <c r="G12" s="35"/>
       <c r="H12" s="35"/>
       <c r="I12" s="29"/>
@@ -2432,21 +2566,23 @@
       <c r="BK12" s="29"/>
       <c r="BL12" s="29"/>
     </row>
-    <row r="13" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="7"/>
+    <row r="13" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4"/>
       <c r="B13" s="37" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="39">
-        <v>0.2</v>
-      </c>
-      <c r="E13" s="40">
+      <c r="D13" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="40" t="n">
         <v>46106</v>
       </c>
-      <c r="F13" s="40"/>
+      <c r="F13" s="40" t="n">
+        <v>46181</v>
+      </c>
       <c r="G13" s="35"/>
       <c r="H13" s="35"/>
       <c r="I13" s="29"/>
@@ -2506,8 +2642,8 @@
       <c r="BK13" s="29"/>
       <c r="BL13" s="29"/>
     </row>
-    <row r="14" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
+    <row r="14" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>27</v>
       </c>
       <c r="B14" s="37" t="s">
@@ -2516,18 +2652,18 @@
       <c r="C14" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="39">
+      <c r="D14" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="40">
+      <c r="E14" s="40" t="n">
         <v>46029</v>
       </c>
-      <c r="F14" s="40">
+      <c r="F14" s="40" t="n">
         <v>46106</v>
       </c>
       <c r="G14" s="35"/>
-      <c r="H14" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H14" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>78</v>
       </c>
       <c r="I14" s="29"/>
@@ -2587,21 +2723,21 @@
       <c r="BK14" s="29"/>
       <c r="BL14" s="29"/>
     </row>
-    <row r="15" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7"/>
+    <row r="15" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4"/>
       <c r="B15" s="37" t="s">
         <v>29</v>
       </c>
       <c r="C15" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="39">
+      <c r="D15" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="40">
+      <c r="E15" s="40" t="n">
         <v>46035</v>
       </c>
-      <c r="F15" s="40">
+      <c r="F15" s="40" t="n">
         <v>46064</v>
       </c>
       <c r="G15" s="35"/>
@@ -2663,21 +2799,21 @@
       <c r="BK15" s="29"/>
       <c r="BL15" s="29"/>
     </row>
-    <row r="16" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="7"/>
+    <row r="16" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4"/>
       <c r="B16" s="37" t="s">
         <v>30</v>
       </c>
       <c r="C16" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="39">
+      <c r="D16" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="40">
+      <c r="E16" s="40" t="n">
         <v>46063</v>
       </c>
-      <c r="F16" s="40">
+      <c r="F16" s="40" t="n">
         <v>46108</v>
       </c>
       <c r="G16" s="35"/>
@@ -2739,21 +2875,21 @@
       <c r="BK16" s="29"/>
       <c r="BL16" s="29"/>
     </row>
-    <row r="17" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="7"/>
+    <row r="17" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4"/>
       <c r="B17" s="37" t="s">
         <v>31</v>
       </c>
       <c r="C17" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D17" s="39">
-        <v>0.7</v>
-      </c>
-      <c r="E17" s="40">
+      <c r="D17" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="40" t="n">
         <v>46106</v>
       </c>
-      <c r="F17" s="40">
+      <c r="F17" s="40" t="n">
         <v>46108</v>
       </c>
       <c r="G17" s="35"/>
@@ -2815,21 +2951,21 @@
       <c r="BK17" s="29"/>
       <c r="BL17" s="29"/>
     </row>
-    <row r="18" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="7"/>
+    <row r="18" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4"/>
       <c r="B18" s="37" t="s">
         <v>32</v>
       </c>
       <c r="C18" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="39">
+      <c r="D18" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="40">
+      <c r="E18" s="40" t="n">
         <v>46063</v>
       </c>
-      <c r="F18" s="40">
+      <c r="F18" s="40" t="n">
         <v>46064</v>
       </c>
       <c r="G18" s="35"/>
@@ -2891,21 +3027,21 @@
       <c r="BK18" s="29"/>
       <c r="BL18" s="29"/>
     </row>
-    <row r="19" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="7"/>
+    <row r="19" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4"/>
       <c r="B19" s="37" t="s">
         <v>33</v>
       </c>
       <c r="C19" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D19" s="39">
+      <c r="D19" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="40">
+      <c r="E19" s="40" t="n">
         <v>46035</v>
       </c>
-      <c r="F19" s="40">
+      <c r="F19" s="40" t="n">
         <v>46064</v>
       </c>
       <c r="G19" s="35"/>
@@ -2967,26 +3103,26 @@
       <c r="BK19" s="29"/>
       <c r="BL19" s="29"/>
     </row>
-    <row r="20" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
+    <row r="20" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1"/>
       <c r="B20" s="37" t="s">
         <v>34</v>
       </c>
       <c r="C20" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D20" s="39">
+      <c r="D20" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="40">
+      <c r="E20" s="40" t="n">
         <v>46035</v>
       </c>
-      <c r="F20" s="40">
+      <c r="F20" s="40" t="n">
         <v>46106</v>
       </c>
       <c r="G20" s="35"/>
-      <c r="H20" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H20" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>72</v>
       </c>
       <c r="I20" s="29"/>
@@ -3046,26 +3182,26 @@
       <c r="BK20" s="29"/>
       <c r="BL20" s="29"/>
     </row>
-    <row r="21" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
+    <row r="21" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1"/>
       <c r="B21" s="37" t="s">
         <v>35</v>
       </c>
       <c r="C21" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="39">
+      <c r="D21" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="40">
+      <c r="E21" s="40" t="n">
         <v>46042</v>
       </c>
-      <c r="F21" s="40">
+      <c r="F21" s="40" t="n">
         <v>46057</v>
       </c>
       <c r="G21" s="35"/>
-      <c r="H21" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H21" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>16</v>
       </c>
       <c r="I21" s="29"/>
@@ -3125,21 +3261,21 @@
       <c r="BK21" s="29"/>
       <c r="BL21" s="29"/>
     </row>
-    <row r="22" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
+    <row r="22" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1"/>
       <c r="B22" s="37" t="s">
         <v>36</v>
       </c>
       <c r="C22" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="39">
+      <c r="D22" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="40">
+      <c r="E22" s="40" t="n">
         <v>46106</v>
       </c>
-      <c r="F22" s="40">
+      <c r="F22" s="40" t="n">
         <v>46106</v>
       </c>
       <c r="G22" s="35"/>
@@ -3201,19 +3337,27 @@
       <c r="BK22" s="29"/>
       <c r="BL22" s="29"/>
     </row>
-    <row r="23" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
+    <row r="23" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1"/>
       <c r="B23" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="C23" s="38"/>
-      <c r="D23" s="39"/>
-      <c r="E23" s="40"/>
-      <c r="F23" s="40"/>
+      <c r="C23" s="38" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="40" t="n">
+        <v>46174</v>
+      </c>
+      <c r="F23" s="40" t="n">
+        <v>46181</v>
+      </c>
       <c r="G23" s="35"/>
-      <c r="H23" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v/>
+      <c r="H23" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>8</v>
       </c>
       <c r="I23" s="29"/>
       <c r="J23" s="29"/>
@@ -3272,21 +3416,29 @@
       <c r="BK23" s="29"/>
       <c r="BL23" s="29"/>
     </row>
-    <row r="24" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="7" t="s">
+    <row r="24" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>38</v>
       </c>
       <c r="B24" s="42" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="43"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="46"/>
+      <c r="C24" s="43" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="45" t="n">
+        <v>46063</v>
+      </c>
+      <c r="F24" s="46" t="n">
+        <v>46085</v>
+      </c>
       <c r="G24" s="35"/>
-      <c r="H24" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v/>
+      <c r="H24" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>23</v>
       </c>
       <c r="I24" s="29"/>
       <c r="J24" s="29"/>
@@ -3345,26 +3497,26 @@
       <c r="BK24" s="29"/>
       <c r="BL24" s="29"/>
     </row>
-    <row r="25" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="7"/>
+    <row r="25" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4"/>
       <c r="B25" s="47" t="s">
         <v>40</v>
       </c>
       <c r="C25" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="49">
+      <c r="D25" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="50">
+      <c r="E25" s="50" t="n">
         <v>46063</v>
       </c>
-      <c r="F25" s="50">
+      <c r="F25" s="50" t="n">
         <v>46078</v>
       </c>
       <c r="G25" s="35"/>
-      <c r="H25" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H25" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>16</v>
       </c>
       <c r="I25" s="29"/>
@@ -3424,26 +3576,26 @@
       <c r="BK25" s="29"/>
       <c r="BL25" s="29"/>
     </row>
-    <row r="26" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
+    <row r="26" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1"/>
       <c r="B26" s="47" t="s">
         <v>41</v>
       </c>
       <c r="C26" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="D26" s="49">
+      <c r="D26" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="50">
+      <c r="E26" s="50" t="n">
         <v>46077</v>
       </c>
-      <c r="F26" s="50">
+      <c r="F26" s="50" t="n">
         <v>46085</v>
       </c>
       <c r="G26" s="35"/>
-      <c r="H26" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H26" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>9</v>
       </c>
       <c r="I26" s="29"/>
@@ -3503,26 +3655,26 @@
       <c r="BK26" s="29"/>
       <c r="BL26" s="29"/>
     </row>
-    <row r="27" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="4"/>
+    <row r="27" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1"/>
       <c r="B27" s="47" t="s">
         <v>42</v>
       </c>
       <c r="C27" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="D27" s="49">
+      <c r="D27" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="50">
+      <c r="E27" s="50" t="n">
         <v>46084</v>
       </c>
-      <c r="F27" s="50">
+      <c r="F27" s="50" t="n">
         <v>46092</v>
       </c>
       <c r="G27" s="35"/>
-      <c r="H27" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H27" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>9</v>
       </c>
       <c r="I27" s="29"/>
@@ -3582,26 +3734,26 @@
       <c r="BK27" s="29"/>
       <c r="BL27" s="29"/>
     </row>
-    <row r="28" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
+    <row r="28" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1"/>
       <c r="B28" s="47" t="s">
         <v>43</v>
       </c>
       <c r="C28" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="D28" s="49">
+      <c r="D28" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="50">
+      <c r="E28" s="50" t="n">
         <v>46105</v>
       </c>
-      <c r="F28" s="50">
+      <c r="F28" s="50" t="n">
         <v>46106</v>
       </c>
       <c r="G28" s="35"/>
-      <c r="H28" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H28" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>2</v>
       </c>
       <c r="I28" s="29"/>
@@ -3661,22 +3813,22 @@
       <c r="BK28" s="29"/>
       <c r="BL28" s="29"/>
     </row>
-    <row r="29" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4"/>
+    <row r="29" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1"/>
       <c r="B29" s="47" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="C29" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="49">
+      <c r="D29" s="49" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="50" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="F29" s="50" t="s">
-        <v>73</v>
+        <v>45</v>
       </c>
       <c r="G29" s="35"/>
       <c r="H29" s="35"/>
@@ -3737,21 +3889,21 @@
       <c r="BK29" s="29"/>
       <c r="BL29" s="29"/>
     </row>
-    <row r="30" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="4"/>
-      <c r="B30" s="53" t="s">
-        <v>44</v>
+    <row r="30" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1"/>
+      <c r="B30" s="47" t="s">
+        <v>46</v>
       </c>
       <c r="C30" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="D30" s="49">
-        <v>0.2</v>
-      </c>
-      <c r="E30" s="50">
+      <c r="D30" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="50" t="n">
         <v>46091</v>
       </c>
-      <c r="F30" s="50">
+      <c r="F30" s="50" t="n">
         <v>46092</v>
       </c>
       <c r="G30" s="35"/>
@@ -3813,21 +3965,29 @@
       <c r="BK30" s="29"/>
       <c r="BL30" s="29"/>
     </row>
-    <row r="31" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B31" s="54" t="s">
-        <v>46</v>
-      </c>
-      <c r="C31" s="55"/>
-      <c r="D31" s="56"/>
-      <c r="E31" s="57"/>
-      <c r="F31" s="58"/>
+    <row r="31" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B31" s="53" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="56" t="n">
+        <v>46063</v>
+      </c>
+      <c r="F31" s="57" t="n">
+        <v>46120</v>
+      </c>
       <c r="G31" s="35"/>
-      <c r="H31" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v/>
+      <c r="H31" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>58</v>
       </c>
       <c r="I31" s="29"/>
       <c r="J31" s="29"/>
@@ -3886,26 +4046,26 @@
       <c r="BK31" s="29"/>
       <c r="BL31" s="29"/>
     </row>
-    <row r="32" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="4"/>
-      <c r="B32" s="59" t="s">
-        <v>47</v>
-      </c>
-      <c r="C32" s="60" t="s">
+    <row r="32" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1"/>
+      <c r="B32" s="58" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="D32" s="61">
+      <c r="D32" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="62">
+      <c r="E32" s="61" t="n">
         <v>46063</v>
       </c>
-      <c r="F32" s="62">
+      <c r="F32" s="61" t="n">
         <v>46071</v>
       </c>
       <c r="G32" s="35"/>
-      <c r="H32" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H32" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>9</v>
       </c>
       <c r="I32" s="29"/>
@@ -3965,26 +4125,26 @@
       <c r="BK32" s="29"/>
       <c r="BL32" s="29"/>
     </row>
-    <row r="33" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="4"/>
-      <c r="B33" s="59" t="s">
-        <v>48</v>
-      </c>
-      <c r="C33" s="60" t="s">
+    <row r="33" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1"/>
+      <c r="B33" s="58" t="s">
+        <v>50</v>
+      </c>
+      <c r="C33" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="D33" s="61">
+      <c r="D33" s="60" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="62">
+      <c r="E33" s="61" t="n">
         <v>46091</v>
       </c>
-      <c r="F33" s="62">
+      <c r="F33" s="61" t="n">
         <v>46092</v>
       </c>
       <c r="G33" s="35"/>
-      <c r="H33" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H33" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>2</v>
       </c>
       <c r="I33" s="29"/>
@@ -4044,23 +4204,27 @@
       <c r="BK33" s="29"/>
       <c r="BL33" s="29"/>
     </row>
-    <row r="34" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="4"/>
-      <c r="B34" s="59" t="s">
-        <v>49</v>
-      </c>
-      <c r="C34" s="60" t="s">
+    <row r="34" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1"/>
+      <c r="B34" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="C34" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="D34" s="61">
-        <v>0</v>
-      </c>
-      <c r="E34" s="63"/>
-      <c r="F34" s="63"/>
+      <c r="D34" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="61" t="n">
+        <v>46117</v>
+      </c>
+      <c r="F34" s="61" t="n">
+        <v>46120</v>
+      </c>
       <c r="G34" s="35"/>
-      <c r="H34" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v/>
+      <c r="H34" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>4</v>
       </c>
       <c r="I34" s="29"/>
       <c r="J34" s="29"/>
@@ -4119,26 +4283,26 @@
       <c r="BK34" s="29"/>
       <c r="BL34" s="29"/>
     </row>
-    <row r="35" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="4"/>
-      <c r="B35" s="59" t="s">
-        <v>50</v>
-      </c>
-      <c r="C35" s="60" t="s">
+    <row r="35" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1"/>
+      <c r="B35" s="58" t="s">
+        <v>52</v>
+      </c>
+      <c r="C35" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="D35" s="61">
-        <v>0.5</v>
-      </c>
-      <c r="E35" s="62">
+      <c r="D35" s="60" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="61" t="n">
         <v>46091</v>
       </c>
-      <c r="F35" s="62">
+      <c r="F35" s="61" t="n">
         <v>46092</v>
       </c>
       <c r="G35" s="35"/>
-      <c r="H35" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H35" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>2</v>
       </c>
       <c r="I35" s="29"/>
@@ -4198,21 +4362,29 @@
       <c r="BK35" s="29"/>
       <c r="BL35" s="29"/>
     </row>
-    <row r="36" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B36" s="64" t="s">
-        <v>51</v>
-      </c>
-      <c r="C36" s="65"/>
-      <c r="D36" s="66"/>
-      <c r="E36" s="67"/>
-      <c r="F36" s="68"/>
+    <row r="36" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36" s="62" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" s="63" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="65" t="n">
+        <v>46054</v>
+      </c>
+      <c r="F36" s="66" t="n">
+        <v>46064</v>
+      </c>
       <c r="G36" s="35"/>
-      <c r="H36" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v/>
+      <c r="H36" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <v>11</v>
       </c>
       <c r="I36" s="29"/>
       <c r="J36" s="29"/>
@@ -4271,26 +4443,26 @@
       <c r="BK36" s="29"/>
       <c r="BL36" s="29"/>
     </row>
-    <row r="37" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="4"/>
-      <c r="B37" s="69" t="s">
-        <v>52</v>
-      </c>
-      <c r="C37" s="70" t="s">
+    <row r="37" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1"/>
+      <c r="B37" s="67" t="s">
+        <v>54</v>
+      </c>
+      <c r="C37" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="D37" s="71">
+      <c r="D37" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="E37" s="72">
+      <c r="E37" s="70" t="n">
         <v>46054</v>
       </c>
-      <c r="F37" s="73">
+      <c r="F37" s="70" t="n">
         <v>46064</v>
       </c>
       <c r="G37" s="35"/>
-      <c r="H37" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H37" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>11</v>
       </c>
       <c r="I37" s="52"/>
@@ -4350,26 +4522,26 @@
       <c r="BK37" s="29"/>
       <c r="BL37" s="29"/>
     </row>
-    <row r="38" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="4"/>
-      <c r="B38" s="69" t="s">
-        <v>53</v>
-      </c>
-      <c r="C38" s="70" t="s">
+    <row r="38" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1"/>
+      <c r="B38" s="67" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" s="68" t="s">
         <v>6</v>
       </c>
-      <c r="D38" s="71">
+      <c r="D38" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="E38" s="73">
+      <c r="E38" s="70" t="n">
         <v>46054</v>
       </c>
-      <c r="F38" s="73">
+      <c r="F38" s="70" t="n">
         <v>46064</v>
       </c>
       <c r="G38" s="35"/>
-      <c r="H38" s="35">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+      <c r="H38" s="35" t="n">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v>11</v>
       </c>
       <c r="I38" s="52"/>
@@ -4429,18 +4601,18 @@
       <c r="BK38" s="29"/>
       <c r="BL38" s="29"/>
     </row>
-    <row r="39" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B39" s="74"/>
-      <c r="C39" s="75"/>
-      <c r="D39" s="76"/>
-      <c r="E39" s="77"/>
-      <c r="F39" s="77"/>
+    <row r="39" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" s="71"/>
+      <c r="C39" s="72"/>
+      <c r="D39" s="73"/>
+      <c r="E39" s="74"/>
+      <c r="F39" s="74"/>
       <c r="G39" s="35"/>
       <c r="H39" s="35" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I39" s="29"/>
@@ -4500,192 +4672,210 @@
       <c r="BK39" s="29"/>
       <c r="BL39" s="29"/>
     </row>
-    <row r="40" spans="1:64" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B40" s="78" t="s">
-        <v>56</v>
-      </c>
-      <c r="C40" s="79"/>
-      <c r="D40" s="80"/>
-      <c r="E40" s="81"/>
-      <c r="F40" s="82"/>
-      <c r="G40" s="83"/>
-      <c r="H40" s="83" t="str">
-        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+    <row r="40" s="36" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B40" s="75" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="76"/>
+      <c r="D40" s="77"/>
+      <c r="E40" s="78"/>
+      <c r="F40" s="79"/>
+      <c r="G40" s="80"/>
+      <c r="H40" s="80" t="str">
+        <f aca="false">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
-      <c r="I40" s="84"/>
-      <c r="J40" s="84"/>
-      <c r="K40" s="84"/>
-      <c r="L40" s="84"/>
-      <c r="M40" s="84"/>
-      <c r="N40" s="84"/>
-      <c r="O40" s="84"/>
-      <c r="P40" s="84"/>
-      <c r="Q40" s="84"/>
-      <c r="R40" s="84"/>
-      <c r="S40" s="84"/>
-      <c r="T40" s="84"/>
-      <c r="U40" s="84"/>
-      <c r="V40" s="84"/>
-      <c r="W40" s="84"/>
-      <c r="X40" s="84"/>
-      <c r="Y40" s="84"/>
-      <c r="Z40" s="84"/>
-      <c r="AA40" s="84"/>
-      <c r="AB40" s="84"/>
-      <c r="AC40" s="84"/>
-      <c r="AD40" s="84"/>
-      <c r="AE40" s="84"/>
-      <c r="AF40" s="84"/>
-      <c r="AG40" s="84"/>
-      <c r="AH40" s="84"/>
-      <c r="AI40" s="84"/>
-      <c r="AJ40" s="84"/>
-      <c r="AK40" s="84"/>
-      <c r="AL40" s="84"/>
-      <c r="AM40" s="84"/>
-      <c r="AN40" s="84"/>
-      <c r="AO40" s="84"/>
-      <c r="AP40" s="84"/>
-      <c r="AQ40" s="84"/>
-      <c r="AR40" s="84"/>
-      <c r="AS40" s="84"/>
-      <c r="AT40" s="84"/>
-      <c r="AU40" s="84"/>
-      <c r="AV40" s="84"/>
-      <c r="AW40" s="84"/>
-      <c r="AX40" s="84"/>
-      <c r="AY40" s="84"/>
-      <c r="AZ40" s="84"/>
-      <c r="BA40" s="84"/>
-      <c r="BB40" s="84"/>
-      <c r="BC40" s="84"/>
-      <c r="BD40" s="84"/>
-      <c r="BE40" s="84"/>
-      <c r="BF40" s="84"/>
-      <c r="BG40" s="84"/>
-      <c r="BH40" s="84"/>
-      <c r="BI40" s="84"/>
-      <c r="BJ40" s="84"/>
-      <c r="BK40" s="84"/>
-      <c r="BL40" s="84"/>
-    </row>
-    <row r="41" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G41" s="85"/>
-    </row>
-    <row r="42" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C42" s="86"/>
-      <c r="F42" s="87"/>
-    </row>
-    <row r="43" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C43" s="88"/>
-    </row>
-    <row r="1048573" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048574" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048575" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1048576" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="I40" s="81"/>
+      <c r="J40" s="81"/>
+      <c r="K40" s="81"/>
+      <c r="L40" s="81"/>
+      <c r="M40" s="81"/>
+      <c r="N40" s="81"/>
+      <c r="O40" s="81"/>
+      <c r="P40" s="81"/>
+      <c r="Q40" s="81"/>
+      <c r="R40" s="81"/>
+      <c r="S40" s="81"/>
+      <c r="T40" s="81"/>
+      <c r="U40" s="81"/>
+      <c r="V40" s="81"/>
+      <c r="W40" s="81"/>
+      <c r="X40" s="81"/>
+      <c r="Y40" s="81"/>
+      <c r="Z40" s="81"/>
+      <c r="AA40" s="81"/>
+      <c r="AB40" s="81"/>
+      <c r="AC40" s="81"/>
+      <c r="AD40" s="81"/>
+      <c r="AE40" s="81"/>
+      <c r="AF40" s="81"/>
+      <c r="AG40" s="81"/>
+      <c r="AH40" s="81"/>
+      <c r="AI40" s="81"/>
+      <c r="AJ40" s="81"/>
+      <c r="AK40" s="81"/>
+      <c r="AL40" s="81"/>
+      <c r="AM40" s="81"/>
+      <c r="AN40" s="81"/>
+      <c r="AO40" s="81"/>
+      <c r="AP40" s="81"/>
+      <c r="AQ40" s="81"/>
+      <c r="AR40" s="81"/>
+      <c r="AS40" s="81"/>
+      <c r="AT40" s="81"/>
+      <c r="AU40" s="81"/>
+      <c r="AV40" s="81"/>
+      <c r="AW40" s="81"/>
+      <c r="AX40" s="81"/>
+      <c r="AY40" s="81"/>
+      <c r="AZ40" s="81"/>
+      <c r="BA40" s="81"/>
+      <c r="BB40" s="81"/>
+      <c r="BC40" s="81"/>
+      <c r="BD40" s="81"/>
+      <c r="BE40" s="81"/>
+      <c r="BF40" s="81"/>
+      <c r="BG40" s="81"/>
+      <c r="BH40" s="81"/>
+      <c r="BI40" s="81"/>
+      <c r="BJ40" s="81"/>
+      <c r="BK40" s="81"/>
+      <c r="BL40" s="81"/>
+    </row>
+    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="G41" s="82"/>
+    </row>
+    <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C42" s="83"/>
+      <c r="F42" s="84"/>
+    </row>
+    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C43" s="85"/>
+    </row>
+    <row r="1048573" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="BF5:BL5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="I5:O5"/>
+    <mergeCell ref="P5:V5"/>
     <mergeCell ref="W5:AC5"/>
     <mergeCell ref="AD5:AJ5"/>
     <mergeCell ref="AK5:AQ5"/>
     <mergeCell ref="AR5:AX5"/>
     <mergeCell ref="AY5:BE5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="I5:O5"/>
-    <mergeCell ref="P5:V5"/>
+    <mergeCell ref="BF5:BL5"/>
   </mergeCells>
-  <conditionalFormatting sqref="D30">
-    <cfRule type="dataBar" priority="18">
-      <dataBar>
+  <conditionalFormatting sqref="I10:BL40">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>AND($C10=$E$3,task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>AND($C10=$D$3,task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>AND($C10=$C$3,task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
+      <formula>AND($C10=$E$3,task_end&gt;=I$6,task_start&lt;=I$6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>AND($C10=$D$3,task_end&gt;=I$6,task_start&lt;=I$6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I10:BL38">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>AND($C10=$C$3,task_end&gt;=I$6,task_start&lt;=I$6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D31:D40 D8:D29">
+    <cfRule type="dataBar" priority="8">
+      <dataBar showValue="1" minLength="10" maxLength="90">
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
         <color rgb="FFBFBFBF"/>
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4F65FC90-AE97-457C-B06F-1953BCF47390}</x14:id>
+          <x14:id>{6ACE4FAC-E61E-436F-8BD8-F0D59CE34A00}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D31:D40 D8:D29">
-    <cfRule type="dataBar" priority="8">
-      <dataBar>
+  <conditionalFormatting sqref="I8:BL40">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>AND(task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>AND(task_end&gt;=I$6,task_start&lt;J$6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:BL40">
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+      <formula>AND(TODAY()&gt;=I$6,TODAY()&lt;J$6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D30">
+    <cfRule type="dataBar" priority="12">
+      <dataBar showValue="1" minLength="10" maxLength="90">
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
         <color rgb="FFBFBFBF"/>
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4EEE73CF-252E-4726-B754-60689BF514AE}</x14:id>
+          <x14:id>{5172C06C-905A-4F4B-8CA6-3A4BC650F3DC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:BL40">
-    <cfRule type="expression" dxfId="8" priority="11">
-      <formula>AND(TODAY()&gt;=I$6,TODAY()&lt;J$6)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I8:BL40">
-    <cfRule type="expression" dxfId="7" priority="9">
-      <formula>AND(task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="10">
-      <formula>AND(task_end&gt;=I$6,task_start&lt;J$6)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10:BL38">
-    <cfRule type="expression" dxfId="5" priority="7">
-      <formula>AND($C10=$C$3,task_end&gt;=I$6,task_start&lt;=I$6)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I10:BL40">
-    <cfRule type="expression" dxfId="4" priority="2">
-      <formula>AND($C10=$E$3,task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>AND($C10=$D$3,task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
-      <formula>AND($C10=$C$3,task_start&lt;=I$6,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="5">
-      <formula>AND($C10=$E$3,task_end&gt;=I$6,task_start&lt;=I$6)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="6">
-      <formula>AND($C10=$D$3,task_end&gt;=I$6,task_start&lt;=I$6)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" promptTitle="Woche anzeigen" prompt="Das Ändern dieser Zahl bewirkt ein Scrollen in der Gantt-Diagrammansicht." sqref="E5" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="greaterThanOrEqual" prompt="Das Ändern dieser Zahl bewirkt ein Scrollen in der Gantt-Diagrammansicht." promptTitle="Woche anzeigen" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="E5" type="whole">
       <formula1>1</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C10:C23 C25:C30 C32:C35 C37:C38" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C10:C23 C25:C30 C32:C35 C37:C38" type="list">
       <formula1>$C$3:$E$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.34722222222222199" header="0.511811023622047" footer="0.3"/>
-  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
-  <headerFooter differentFirst="1">
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.347222222222222" header="0.511811023622047" footer="0.3"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="true" differentOddEven="false">
+    <oddHeader/>
     <oddFooter>&amp;CPage &amp;P of &amp;N</oddFooter>
+    <firstHeader/>
+    <firstFooter/>
   </headerFooter>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4F65FC90-AE97-457C-B06F-1953BCF47390}">
-            <x14:dataBar gradient="0">
+          <x14:cfRule type="dataBar" id="{6ACE4FAC-E61E-436F-8BD8-F0D59CE34A00}">
+            <x14:dataBar minLength="10" maxLength="90" axisPosition="automatic" gradient="false">
+              <x14:cfvo type="num">
+                <xm:f>0</xm:f>
+              </x14:cfvo>
+              <x14:cfvo type="num">
+                <xm:f>1</xm:f>
+              </x14:cfvo>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>D31:D40 D8:D29</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{5172C06C-905A-4F4B-8CA6-3A4BC650F3DC}">
+            <x14:dataBar minLength="10" maxLength="90" axisPosition="automatic" gradient="false">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
               </x14:cfvo>
@@ -4698,21 +4888,6 @@
           </x14:cfRule>
           <xm:sqref>D30</xm:sqref>
         </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4EEE73CF-252E-4726-B754-60689BF514AE}">
-            <x14:dataBar gradient="0">
-              <x14:cfvo type="num">
-                <xm:f>0</xm:f>
-              </x14:cfvo>
-              <x14:cfvo type="num">
-                <xm:f>1</xm:f>
-              </x14:cfvo>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>D31:D40 D8:D29</xm:sqref>
-        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>
@@ -4720,101 +4895,109 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.5" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="13.5" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="87.16796875" style="89" customWidth="1"/>
-    <col min="2" max="16384" width="9.14453125" style="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="86" width="87.17"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="2" style="7" width="9.14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="1:2" s="91" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A2" s="90" t="s">
-        <v>57</v>
-      </c>
-      <c r="B2" s="90"/>
-    </row>
-    <row r="3" spans="1:2" s="94" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="92" t="s">
-        <v>58</v>
-      </c>
-      <c r="B3" s="93"/>
-    </row>
-    <row r="4" spans="1:2" s="96" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A4" s="95" t="s">
+    <row r="1" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="2" s="88" customFormat="true" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="87" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="73.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="97" t="s">
+      <c r="B2" s="87"/>
+    </row>
+    <row r="3" s="91" customFormat="true" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="89" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="95" t="s">
+      <c r="B3" s="90"/>
+    </row>
+    <row r="4" s="93" customFormat="true" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="92" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="89" customFormat="1" ht="204.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="98" t="s">
+    <row r="5" customFormat="false" ht="73.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="94" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="96" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A8" s="95" t="s">
+    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="92" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="68.25" x14ac:dyDescent="0.2">
-      <c r="A9" s="97" t="s">
+    <row r="7" s="86" customFormat="true" ht="204.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="95" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="89" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="99" t="s">
+    <row r="8" s="93" customFormat="true" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="92" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="96" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="95" t="s">
+    <row r="9" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="94" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="27.75" x14ac:dyDescent="0.2">
-      <c r="A12" s="97" t="s">
+    <row r="10" s="86" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="96" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="89" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="99" t="s">
+    <row r="11" s="93" customFormat="true" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="92" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="14" spans="1:2" s="96" customFormat="1" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A14" s="95" t="s">
+    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="94" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="97" t="s">
+    <row r="13" s="86" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="96" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="68.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="97" t="s">
+    <row r="14" s="93" customFormat="true" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="92" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="94" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="94" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
-    <hyperlink ref="A10" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
-    <hyperlink ref="A13" r:id="rId4" xr:uid="{00000000-0004-0000-0100-000003000000}"/>
+    <hyperlink ref="A2" r:id="rId1" display="EINFACHES GANTT-DIAGRAMM von Vertex42.com"/>
+    <hyperlink ref="A3" r:id="rId2" display="https://www.vertex42.com/ExcelTemplates/simple-gantt-chart.html"/>
+    <hyperlink ref="A10" r:id="rId3" display="Verwenden des einfachen Gantt-Diagramms"/>
+    <hyperlink ref="A13" r:id="rId4" display="Projektmanagementvorlagen"/>
   </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.5" right="0.5" top="0.5" bottom="0.5" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
   <drawing r:id="rId5"/>
 </worksheet>
 </file>

</xml_diff>